<commit_message>
implementacion en ollama y ragas para la evaluación
</commit_message>
<xml_diff>
--- a/backend/evaluation/metrics.xlsx
+++ b/backend/evaluation/metrics.xlsx
@@ -425,28 +425,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>question</t>
+          <t>user_input</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>ground_truth</t>
+          <t>retrieved_contexts</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>new_answer</t>
+          <t>response</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>context</t>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>context_precision</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>context_recall</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>faithfulness</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>answer_relevancy</t>
         </is>
       </c>
     </row>
@@ -458,7 +478,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>To assess changes in reproductive, maternal, newborn, child, and adolescent health (RMNCAH) indicators in Haiti from August 2018 to September 2021, before and during COVID-19.</t>
+          <t>['To achieve the objective of the study, the analysis was divided into two periods: pre- and peri-COVID-19 pandemic. Pre-COVID-19 pandemic included the first 19 months before the report of the first COVID-19 case in Haiti (– ); and peri-COVID-19, the 19 months starting from the detection of the first case (–). Two sample t-tests for proportions were used to compare the frequency of indicators before and during the COVID-19 pan- demic. Analyses for reproductive and maternal indicators were disaggregated by age, and neonatal and child health indicators were disaggregated by sex wherever possible. for indicators with unknown denominator (unavailable in SISNU to calculate proportion), we relied on data from the Haitian Institute of Sta- tistics and', 'Joseph et al. « COVID-19 and reproductive, maternal, and child health in Haiti\n\nOriginal research\n\nsignificance level was defined at less than 0.05. All the analyses were carried out using Microsoft Excel and Stata (Stata Statisti- cal Software, Release 14, 2015; StataCorp, College Station, TX).\n\nRESULTS', 'ABSTRACT Objective. To assess changes in reproductive, maternal, newborn, child, and adolescent health (RMNCAH) in Haiti from to , before and during the COVID-19 pandemic.\n\nMethods. A retrospective study using surveillance data from the Haitian Unique Health Information System, examining two periods: pre- and peri-COVID-19 pandemic. Health indicators at the national level in the two periods were compared using two-sample t-tests for proportions, and average absolute monthly changes were calculated using variance-weighted regression.', 'This study included all women of reproductive age (15–49 years) who had their information on reproductive and mater- nal health/death recorded on the above-mentioned databases from to . The study also included newborns, under-5 children, and adolescents for which infor- mation was available for the same periods. All the data used in this study were anonymized to ensure the confidentiality of the participants. Ethical approval was obtained from the National Ethics Committee of the Ministry of Health of Haiti prior conducting the study. Participants provided verbal informed consent prior to data collection.', 'Immediately after the report of the first COVID-19 case in in Haiti, the Government put several preventive measures in place to limit the spread of the virus in the coun- try (5, 6). Among these was the creation of the Multisectoral Commission for the Management of the COVID-19 Pandemic, to lead the strategic planning and response against COVID-19 (5, 6). Despite the measures adopted by the Government to limit the spread of the virus, low compliance to the measures by the population was reported (7). Given the fragile health system and poor health indicators in Haiti, it was predicted that dis- ruptions to health services in Haiti could leave 212 600 children without diphtheria, tetanus, and pertussis (DTaP) vaccina- tion, and leads? to 26 500 fewer deliveries in health facilities']</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -469,9 +489,13 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>To assess changes in reproductive, maternal, newborn, child, and adolescent health (RMNCAH) indicators in Haiti from August 2018 to September 2021, before and during COVID-19.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -481,20 +505,23 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>['Data analysis', 'A retrospective study was conducted using data from the Haitian Unique Health Information System (Système d’Infor- mation Sanitaire Unique – SISNU in French). SISNU is a national health information platform launched by the Ministry of Health of Haiti to track all health-related data on RMNCAH in the country on a monthly basis. SISNU captures health-related data from more than 800 facilities from the nation’s 10 depart- ments. The monthly reporting rate for the departments on patient attendance and outpatient clinics is estimated to be over 70%. SISNU collects data on several RMNCAH indicators that can be disaggregated by age and sex. Data collected by SISNU are periodically uploaded to the District Health Information Software 2 (DHIS2), a web-based platform that is being used by 73', 'more than 800 health facilities distributed in the 10 geographic departments, with a monthly reporting rate of over 70%. The analyses were disaggregated by age, and by sex when appli- cable. However, in terms of limitations, our analyses relied on secondary data from SISNU–DHIS2, which may include inaccurate and incomplete reporting, as frequently found in low- and middle-income countries (25, 26). for example, we were unable to distinguish between missing data and true zero values. Nonetheless, in this analysis, the only variable with missing data was the pneumococcal conjugate vaccine indi- cator, which had a 5% missing rate during the pre-COVID-19 pandemic period. We believe that this level of missing data would likely have minimal or negligible impact on the study’s results. Moreover,', 'Source: Prepared by the authors based on DHIS2 data.', 'This study included all women of reproductive age (15–49 years) who had their information on reproductive and mater- nal health/death recorded on the above-mentioned databases from to . The study also included newborns, under-5 children, and adolescents for which infor- mation was available for the same periods. All the data used in this study were anonymized to ensure the confidentiality of the participants. Ethical approval was obtained from the National Ethics Committee of the Ministry of Health of Haiti prior conducting the study. Participants provided verbal informed consent prior to data collection.']</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>The data system used for the analysis was the **Haitian Unique Health Information System (SISNU)**, which is linked to the **District Health Information Software 2 (DHIS2)**. SISNU is a national health information platform that tracks health-related data on reproductive, maternal, newborn, child, and adolescent health (RMNCAH) in Haiti.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>The study used data from the Haitian Unique Health Information System (Système d’Information Sanitaire Unique – SISNU), which is a national health information platform launched in 2013 by the Ministry of Health of Haiti. SISNU data are periodically uploaded to the District Health Information Software 2 (DHIS2) platform for analysis</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>The data system used for the analysis was the **Haitian Unique Health Information System (SISNU)**, which collects data that are periodically uploaded to the **District Health Information Software 2 (DHIS2)**.
-This is stated in the text: "A retrospective study was conducted using data from the Haitian Unique Health Information System (Système d’Infor- mation Sanitaire Unique – SISNU in French)... SISNU collects data on several RMNCAH indicators that can be disaggregated by age and sex... Data collected by SISNU are periodically uploaded to the District Health Information Software 2 (DHIS2)" (Page 2)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -504,22 +531,25 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>['To achieve the objective of the study, the analysis was divided into two periods: pre- and peri-COVID-19 pandemic. Pre-COVID-19 pandemic included the first 19 months before the report of the first COVID-19 case in Haiti (– ); and peri-COVID-19, the 19 months starting from the detection of the first case (–). Two sample t-tests for proportions were used to compare the frequency of indicators before and during the COVID-19 pan- demic. Analyses for reproductive and maternal indicators were disaggregated by age, and neonatal and child health indicators were disaggregated by sex wherever possible. for indicators with unknown denominator (unavailable in SISNU to calculate proportion), we relied on data from the Haitian Institute of Sta- tistics and', 'ABSTRACT Objective. To assess changes in reproductive, maternal, newborn, child, and adolescent health (RMNCAH) in Haiti from to , before and during the COVID-19 pandemic.\n\nMethods. A retrospective study using surveillance data from the Haitian Unique Health Information System, examining two periods: pre- and peri-COVID-19 pandemic. Health indicators at the national level in the two periods were compared using two-sample t-tests for proportions, and average absolute monthly changes were calculated using variance-weighted regression.', 'Metodología. Estudio retrospectivo basado en datos de vigilancia del sistema único de información de salud de Haití para estudiar los periodos pre y peripandémico. La comparación de los indicadores de salud a nivel nacional de estos dos periodos se realizó mediante pruebas de t de dos muestras para comparar propor- ciones, y se calculó el promedio de la variación mensual absoluta mediante una regresión ponderada por la varianza.', 'Our study has strengths and limitations. As strengths, we were able to use a long period to compare the indirect impact of COVID-19 on several RMNCAH indicators nationally. We con- sidered that such a period was sufficient to assess time trends in the indicators and see the effect of public health measures on limiting the spread of the virus. We used data collected from', 'We showed the overall changes in RMNCAH indicators during the first 19 months following the first reported COVID-19 case in Haiti compared with the previous 19 months. Most of the indicators analyzed declined from the pre- to the peri-COVID-19 pandemic period. However, the most affected indicators were for antenatal care and childhood immunization. Indicators such as the proportions of pregnant women with four antenatal care vis- its, pregnant women with five antenatal care visits or more, and pregnant women who received a second dose of tetanus vaccine (dT2+) declined by over 4 percentage points from the pre- to the peri-COVID-19 pandemic period. Likewise, the proportions of children who received BCG, DTaP, polio, pentavalent, and rota- virus vaccines all declined by over 8 percentage']</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>**Two-sample t-tests for proportions** were used to compare the frequency of indicators before and during the COVID-19 pandemic. Additionally, **variance-weighted regression** was used to calculate the average absolute monthly changes in health indicators between the two periods.
+This is stated in the abstract: "Health indicators at the national level in the two periods were compared using two-sample t-tests for proportions, and average absolute monthly changes were calculated using variance-weighted regression." (Page 1)
+And also mentioned in the methodology: "Two sample t-tests for proportions were used to compare the frequency of indicators before and during the COVID-19 pandemic." (Page 2)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Two-sample t-tests for proportions and variance-weighted regression for average absolute monthly changes.</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>The statistical methods applied to compare pre- and peri-COVID-19 periods were:
-* **Two-sample t-tests for proportions**: used to compare the frequency of indicators before and during the COVID-19 pandemic.
-* **Variance-weighted regression**: used to calculate the average absolute monthly changes in health indicators.
-This is stated in the text: "Two sample t-tests for proportions were used to compare the frequency of indicators before and during the COVID-19 pandemic... and average absolute monthly changes were calculated using variance-weighted regression." (Page 2 and Page 1)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -529,25 +559,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>['Maternal health indicators included number of antenatal care visits during pregnancy, number of pregnant women with con- firmed malaria and treated with chloroquine, and with anemia and treated for iron deficiency anemia. Also included were the number of pregnant women who received at least the second dose of tetanus toxoid vaccine (dT2+), number of institutional deliveries and deliveries by C-section, and number of women receiving post-abortion care.\n\nNewborn and postnatal health indicators included: number of home visits/postnatal follow-up (0–3 days) after delivery, low birthweight (&lt;2.5 kg), number of institutional live births beneficiaries of the kangaroo mother care method, and number of institutional live births with early initiation of breastfeeding.', 'Results. There was a statistically significant decline in the proportion of most of the indicators assessed from the pre- to the peri-COVID-19 pandemic period. However, the most affected indicators were the proportions of pregnant women with four antenatal care visits, with five antenatal care visits or more, and those who received a second dose of tetanus vaccine, which decreased by over 4 percentage points during the two periods. Likewise, the proportions of children who received diphtheria, tetanus, and pertussis (DTaP), BCG, polio, pentavalent, and rotavirus vaccines also all declined by over 8 percentage points. in contrast, pneu- mococcal conjugate vaccine increased by over 4 percentage points. A statistically significant decrease was also observed in the average absolute monthly', 'Figure 1 presents the evolution of the maternal mortality ratio during the two periods. The maternal mortality ratio decreased slightly from 195.0 in to 183.0 per 100 000 live births in . The highest ratio was observed in (372.4 per 100 000 live births) and in (356.6 per 100 000 live births). During the peri-COVID-19 pandemic, it increased from 179.6 in to 185.9 per 100 000 live births in .\n\nDISCUSSION', 'We showed the overall changes in RMNCAH indicators during the first 19 months following the first reported COVID-19 case in Haiti compared with the previous 19 months. Most of the indicators analyzed declined from the pre- to the peri-COVID-19 pandemic period. However, the most affected indicators were for antenatal care and childhood immunization. Indicators such as the proportions of pregnant women with four antenatal care vis- its, pregnant women with five antenatal care visits or more, and pregnant women who received a second dose of tetanus vaccine (dT2+) declined by over 4 percentage points from the pre- to the peri-COVID-19 pandemic period. Likewise, the proportions of children who received BCG, DTaP, polio, pentavalent, and rota- virus vaccines all declined by over 8 percentage', 'Finally, the maternal mortality ratio showed a statistically significant increase from 195 to 230 per 100 000 live births from the pre- to the peri-COVID-19 pandemic period (p = 0.0082). The stillbirth rate also increased from 24.4 to 27.1 per 1 000 births during the same period.']</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>The maternal health indicators that saw the most significant decline were:
+1. **Pregnant women with four antenatal care visits**
+2. **Pregnant women with five antenatal care visits or more**
+3. **Pregnant women who received a second dose of tetanus vaccine (dT2+)** 
+These indicators decreased by over 4 percentage points during the pre- and peri-COVID-19 pandemic periods. (Page 4) 
+Additionally, the maternal mortality ratio also showed a statistically significant increase from 195 to 230 per 100,000 live births from the pre- to the peri-COVID-19 pandemic period. (Page 4)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Pregnant women with 4 or more antenatal visits and those receiving the second dose of the tetanus vaccine, each decreasing by more than 4 percentage points.</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>The maternal health indicators that saw the most significant decline were:
-* **Antenatal care visits**: Specifically, the proportions of pregnant women with:
-	+ Four antenatal care visits
-	+ Five antenatal care visits or more
-* **Tetanus vaccination**: The proportion of pregnant women who received a second dose of tetanus vaccine (dT2+)
-These indicators declined by over 4 percentage points from the pre- to the peri-COVID-19 pandemic period.
-This is stated in the text: "However, the most affected indicators were the proportions of pregnant women with four antenatal care visits, with five antenatal care visits or more, and those who received a second dose of tetanus vaccine, which decreased by over 4 percentage points during the two periods." (Page 1) and "Indicators such as the proportions of pregnant women with four antenatal care visits, pregnant women with five antenatal care visits or more, and pregnant women who received a second dose of tetanus vaccine (dT2+) declined by over 4 percentage points from the pre- to the peri-COVID-19 pandemic period." (Page 4)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -557,26 +590,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>['Results. There was a statistically significant decline in the proportion of most of the indicators assessed from the pre- to the peri-COVID-19 pandemic period. However, the most affected indicators were the proportions of pregnant women with four antenatal care visits, with five antenatal care visits or more, and those who received a second dose of tetanus vaccine, which decreased by over 4 percentage points during the two periods. Likewise, the proportions of children who received diphtheria, tetanus, and pertussis (DTaP), BCG, polio, pentavalent, and rotavirus vaccines also all declined by over 8 percentage points. in contrast, pneu- mococcal conjugate vaccine increased by over 4 percentage points. A statistically significant decrease was also observed in the average absolute monthly', 'The proportion of fully vaccinated children (0–11 months) decreased from 48.9% to 46.8% (p &lt; 0.001). However, when the data were disaggregated by sex, these proportions seemed to decrease for female but increase for male children. We believe that such difference could be random and not due to a real difference between males and females in access to vaccination services in the country. The proportion of children aged 6–23 months who received a third dose of vitamin A increased from 1.7% to 2.1% (p &lt; 0.001) and aged 24–59 months, from 2.0% to 2.2% (p &lt; 0.001). There was a slight reduction in the proportion of under-5 children seen for the first time, screened for acute malnutrition (from 12.6% to 12.3%, p &lt; 0.001) as well as for chronic malnutrition (from 3.5% to 3.0%, p &lt; 0.001) ().', 'We showed the overall changes in RMNCAH indicators during the first 19 months following the first reported COVID-19 case in Haiti compared with the previous 19 months. Most of the indicators analyzed declined from the pre- to the peri-COVID-19 pandemic period. However, the most affected indicators were for antenatal care and childhood immunization. Indicators such as the proportions of pregnant women with four antenatal care vis- its, pregnant women with five antenatal care visits or more, and pregnant women who received a second dose of tetanus vaccine (dT2+) declined by over 4 percentage points from the pre- to the peri-COVID-19 pandemic period. Likewise, the proportions of children who received BCG, DTaP, polio, pentavalent, and rota- virus vaccines all declined by over 8 percentage', 'points during the same period. The only indicator that increased by more than 4 percentage points during the period was for pneumococcal conjugate vaccine.', 'Child health indicators analyzed were: total BCG doses (0–11 months), DTaP doses (12–23 months), measles 2 doses (12–23 months), pneumococcal conjugate vaccine 3 doses (0–11 months), polio 3 doses (0–11 months), pentavalent vaccine 3 doses (0–11 months), rotavirus 2 doses (0–11 months), and total fully vaccinated (0–11 months). Child health indicators were disaggregated by sex. It should be noted that most of the vaccine indicators were only available for 0–11 months.\n\nMortality indicators such as the number of maternal deaths per childbirth and number of stillbirths were also analyzed. More details about the indicators and their definition can be found in other resources (9, 10). This study is reported accord- ing to STROBE guidelines for observational studies (11).']</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>The child vaccination indicators that declined the most were:
+1. **BCG (Bacillus Calmette-Guérin) vaccine**
+2. **DTaP (Diphtheria, Tetanus, and Pertussis) vaccine**
+3. **Polio vaccine**
+4. **Pentavalent vaccine**
+5. **Rotavirus vaccine**
+These indicators declined by over 8 percentage points during the pre- and peri-COVID-19 pandemic periods. (Page 4)
+In contrast, the **pneumococcal conjugate vaccine** increased by over 4 percentage points. (Page 4)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>DTaP, BCG, polio, pentavalent, and rotavirus vaccines, all falling by over 8 percentage points.</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>The child vaccination indicators that declined the most were:
-* **Diphtheria, tetanus, and pertussis (DTaP) vaccine**
-* **BCG vaccine**
-* **Polio vaccine**
-* **Pentavalent vaccine**
-* **Rotavirus vaccine**
-These indicators declined by over 8 percentage points from the pre- to the peri-COVID-19 pandemic period.
-This is stated in the text: "Likewise, the proportions of children who received diphtheria, tetanus, and pertussis (DTaP), BCG, polio, pentavalent, and rotavirus vaccines also all declined by over 8 percentage points." (Page 1) and "Likewise, the proportions of children who received BCG, DTaP, polio, pentavalent, and rota- virus vaccines all declined by over 8 percentage points during the same period." (Page 4)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -586,22 +623,23 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>['The number of women opting for the contraceptive implant and children receiving a third dose of pneumococcal con- jugate vaccine increased significantly from the pre- to the peri-COVID-19 pandemic period. This result is, in part, con- sistent with findings from a study by Karp et al. (17) who, using longitudinal data collected from women at risk of unin- tended pregnancy in sub-Saharan Africa during the pre- and peri-COVID-19 pandemic periods, showed that most women did not change contraceptive status in the early months of the pandemic, and those who did were more likely to adopt', 'points during the same period. The only indicator that increased by more than 4 percentage points during the period was for pneumococcal conjugate vaccine.', 'contraception than to discontinue. On the other hand, the increase observed in Haiti in the number of children who received a third dose of pneumococcal conjugate vaccine may be explained by the fact that this vaccine was recently intro- duced into the Government’s routine immunization program (18). Thus, the Government might be more motivated to distribute the new vaccine and vaccinate as many children as possible. However, our results show that the proportion of children aged 0–11 months that were fully vaccinated decreased significantly by 2.1 percentage points from the pre- to the peri- COVID-19 pandemic period.', 'Results. There was a statistically significant decline in the proportion of most of the indicators assessed from the pre- to the peri-COVID-19 pandemic period. However, the most affected indicators were the proportions of pregnant women with four antenatal care visits, with five antenatal care visits or more, and those who received a second dose of tetanus vaccine, which decreased by over 4 percentage points during the two periods. Likewise, the proportions of children who received diphtheria, tetanus, and pertussis (DTaP), BCG, polio, pentavalent, and rotavirus vaccines also all declined by over 8 percentage points. in contrast, pneu- mococcal conjugate vaccine increased by over 4 percentage points. A statistically significant decrease was also observed in the average absolute monthly', 'BCG, bacillus Calmette–Guérin; DTaP, diphtheria, tetanus, and pertussis; PCV, pneumococcal conjugate vaccine. Note: a This variable had 5% missing during the pre-COVID-19 period.\n\nSource: Prepared by the authors based on DHIS2 data.']</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>The **pneumococcal conjugate vaccine** unexpectedly increased during the pandemic. According to the text, it increased by over 4 percentage points during the pre- and peri-COVID-19 pandemic periods (Page 4). This increase may be attributed to the fact that it was recently introduced into the Government's routine immunization program (Page 5).</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>Pneumococcal conjugate vaccine, which rose by more than 4 percentage points.</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>The vaccine that unexpectedly increased during the pandemic was:
-* **Pneumococcal conjugate vaccine**
-This is stated in the text: "Likewise, the proportions of children who received ... pneumococcal conjugate vaccine increased by over 4 percentage points." (Page 1) and "The only indicator that increased by more than 4 percentage points during the period was for pneumococcal conjugate vaccine." (Page 4)
-Additionally, it is noted that this increase may be due to the recent introduction of the vaccine into the Government's routine immunization program, leading to a greater motivation to distribute and administer the vaccine. (Page 5)</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -611,24 +649,23 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>['Finally, the maternal mortality ratio showed a statistically significant increase from 195 to 230 per 100 000 live births from the pre- to the peri-COVID-19 pandemic period (p = 0.0082). The stillbirth rate also increased from 24.4 to 27.1 per 1 000 births during the same period.', 'Figure 1 presents the evolution of the maternal mortality ratio during the two periods. The maternal mortality ratio decreased slightly from 195.0 in to 183.0 per 100 000 live births in . The highest ratio was observed in (372.4 per 100 000 live births) and in (356.6 per 100 000 live births). During the peri-COVID-19 pandemic, it increased from 179.6 in to 185.9 per 100 000 live births in .\n\nDISCUSSION', 'The maternal mortality ratio also increased significantly during the COVID-19 pandemic. This finding is in line with the observations made by de Carvalho et al. (19) in Bahia, Brazil, indicating a marked rise in the maternal mortality ratio during\n\nthe COVID-19 pandemic (19). Such increase might result from maternal illness directly linked to COVID-19 infection, or to the indirect consequence of disruptions in health services and other secondary effects induced by the pandemic.', 'the overwhelming effects of the COVID-19 pandemic could leads? to 31% additional maternal and newborn deaths due to reduced access to essential services such as family planning, antenatal care, facility-based deliveries, and postnatal care (3). in contrast, a retrospective review conducted in Ireland by McDonnell et al. (4) using data from a large tertiary hospital in Dublin found no correlation between the monthly number of COVID-19 deaths and the monthly number of perinatal deaths, preterm births, and hypertensive pregnancies. How- ever, it should be noted that the study focused on severity of the pandemic using the number of COVID-19 deaths as a marker instead of the COVID-19 infection rate (4).', '5000 400.0 4000 300.0 3000 200.0 2000 1000 100.0 Deaths per 100,000 livebirths Absolute number of COVID 19 cases g g . 2019 5 2019 2019 % L i 2020 — ) i 3 ist, 2018 ", £} i, 2019 S r, 2019 A 3 2 r, 2020 . March, 2019 Apri May, 2019 June, July, 2019 3 g June, 2020 July, 2020 — June, 2021 July, 2021 — Augu October, 2018 January, 2019 February, August, October, 2019 January, 2020 August, October, 2020 = August, 2021 — September November, 2018 December, 2018 September November, 2019 December, 2019 September September, 2021 COVID 19 cases o~ Maternal mortality ratio']</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>The maternal mortality ratio showed a statistically significant increase during the peri-COVID-19 period. Specifically, it increased from 195 to 230 per 100,000 live births (Page 4). This increase is also supported by other findings, which suggest that the maternal mortality ratio increased from 179.6 to 185.9 per 100,000 live births during the peri-COVID-19 pandemic period (Page 4). The increase in maternal mortality may be attributed to disruptions in health services, such as reduced access to essential services like family planning, antenatal care, facility-based deliveries, and postnatal care (Page 2).</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>It increased from 195 to 230 deaths per 100,000 live births.</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Maternal mortality increased during the peri-COVID-19 period. 
-The maternal mortality ratio showed a statistically significant increase from 195 to 230 per 100,000 live births (p = 0.0082) from the pre- to the peri-COVID-19 pandemic period. This is supported by findings that the COVID-19 pandemic led to a marked rise in the maternal mortality ratio, possibly due to disruptions in health services and other secondary effects induced by the pandemic.
-This information is stated in the text: 
-"The maternal mortality ratio showed a statistically significant increase from 195 to 230 per 100 000 live births from the pre- to the peri-COVID-19 pandemic period (p = 0.0082)." (Page 4) 
-and 
-"The maternal mortality ratio also increased significantly during the COVID-19 pandemic." (Page 5)</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -638,23 +675,23 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>['offer effective contraception over an extended duration without necessitating frequent visits to healthcare facilities. Alterations in labor and delivery procedures within certain healthcare environments may have led hospitals to adopt new protocols aimed at limiting access to labor-inducing methods, like walking or hydrotherapy, while increasing reliance on surgical interventions such as C-sections. Addi- tionally, expectant mothers may have been more predisposed to choose C-section out of concern for contracting COVID-19 in a hospital environment. The complete lockdown imple- mented by the Government in in response to the swift spread of COVID-19 in other countries, alongside con- cerns about the risk of COVID-19 infection in facilities also treating COVID-19 patients, could', 'There were also reductions in the proportion of institutional delivery (from 69.2% to 67.7%, p &lt; 0.001) and vaginal delivery (from 76.3% to 74.0%, p &lt; 0.001). When institutional delivery was disaggregated by age, no significant differences were observed for adolescent women younger than 15 years and for those aged 15–19 (p &gt; 0.05). On the contrary, the C-section rate increased from 17.5% to 20.2% (p &lt; 0.001) during the same period .', 'When we assessed the time trends in RMNCAH indica- tors with statistically significant AAMC (p &lt; 0.05) during the COVID-19 pandemic, several dips were observed, particu- larly coinciding with the peaks of COVID-19 in the country (May–, –, and May– ).\n\nOnly a small number of indicators, such as the use of intrauterine devices and rate of C-section, increased during the pandemic. An increase in intrauterine device demand during the pandemic might be attributed to the likelihood of women seeking long-acting reversible contraceptives, which', 'the overwhelming effects of the COVID-19 pandemic could leads? to 31% additional maternal and newborn deaths due to reduced access to essential services such as family planning, antenatal care, facility-based deliveries, and postnatal care (3). in contrast, a retrospective review conducted in Ireland by McDonnell et al. (4) using data from a large tertiary hospital in Dublin found no correlation between the monthly number of COVID-19 deaths and the monthly number of perinatal deaths, preterm births, and hypertensive pregnancies. How- ever, it should be noted that the study focused on severity of the pandemic using the number of COVID-19 deaths as a marker instead of the COVID-19 infection rate (4).', 'The number of women opting for the contraceptive implant and children receiving a third dose of pneumococcal con- jugate vaccine increased significantly from the pre- to the peri-COVID-19 pandemic period. This result is, in part, con- sistent with findings from a study by Karp et al. (17) who, using longitudinal data collected from women at risk of unin- tended pregnancy in sub-Saharan Africa during the pre- and peri-COVID-19 pandemic periods, showed that most women did not change contraceptive status in the early months of the pandemic, and those who did were more likely to adopt']</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>The C-section rate increased during the COVID-19 pandemic. According to the text, it increased from 17.5% to 20.2% (p &lt; 0.001) during the same period (Page 4). This trend may be attributed to alterations in labor and delivery procedures, with hospitals adopting new protocols aimed at limiting access to labor-inducing methods and increasing reliance on surgical interventions like C-sections (Page 6). Additionally, expectant mothers may have opted for C-sections due to concerns about contracting COVID-19 in hospital environments (Page 6).</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>The C-section rate increased from 17.5% to 20.2%.</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>The trend observed in C-section deliveries during COVID-19 was an increase. 
-The C-section rate increased from 17.5% to 20.2% (p &lt; 0.001) during the pandemic period. This information is stated in the text: 
-"When institutional delivery was disaggregated by age, no significant differences were observed for adolescent women younger than 15 years and for those aged 15–19 (p &gt; 0.05). On the contrary, the C-section rate increased from 17.5% to 20.2% (p &lt; 0.001) during the same period." (Page 4)
-Additionally, it is noted that alterations in labor and delivery procedures, lockdown implementation, and concerns about COVID-19 infection in hospital environments may have contributed to this increase. (Page 6) 
-The increase in C-section rate is also mentioned in other parts of the text: "Only a small number of indicators, such as the use of intrauterine devices and rate of C-section, increased during the pandemic." (Page 5)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -664,26 +701,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>['We showed the overall changes in RMNCAH indicators during the first 19 months following the first reported COVID-19 case in Haiti compared with the previous 19 months. Most of the indicators analyzed declined from the pre- to the peri-COVID-19 pandemic period. However, the most affected indicators were for antenatal care and childhood immunization. Indicators such as the proportions of pregnant women with four antenatal care vis- its, pregnant women with five antenatal care visits or more, and pregnant women who received a second dose of tetanus vaccine (dT2+) declined by over 4 percentage points from the pre- to the peri-COVID-19 pandemic period. Likewise, the proportions of children who received BCG, DTaP, polio, pentavalent, and rota- virus vaccines all declined by over 8 percentage', 'Results. There was a statistically significant decline in the proportion of most of the indicators assessed from the pre- to the peri-COVID-19 pandemic period. However, the most affected indicators were the proportions of pregnant women with four antenatal care visits, with five antenatal care visits or more, and those who received a second dose of tetanus vaccine, which decreased by over 4 percentage points during the two periods. Likewise, the proportions of children who received diphtheria, tetanus, and pertussis (DTaP), BCG, polio, pentavalent, and rotavirus vaccines also all declined by over 8 percentage points. in contrast, pneu- mococcal conjugate vaccine increased by over 4 percentage points. A statistically significant decrease was also observed in the average absolute monthly', 'presents the newborn and child health indicators during the pre- and peri-COVID-19 pandemic periods. Statisti- cally significant decreases were observed in the proportions of early initiation of breastfeeding among institutional live births (from 60.0% to 58.6%, p &lt; 0.001) and low birthweight (from 11.1% to 10.9%, p = 0.0078). However, there were statistically sig- nificantly increases during the same period in the proportion of institutional live births beneficiaries of the kangaroo mother care method (from 8.6% to 10.4%, p &lt; 0.001) and home visits/postna- tal follow-up during days 0–3 (from 36.8% to 40.0%, p &lt; 0.001).', 'When we assessed the time trends in RMNCAH indica- tors with statistically significant AAMC (p &lt; 0.05) during the COVID-19 pandemic, several dips were observed, particu- larly coinciding with the peaks of COVID-19 in the country (May–, –, and May– ).\n\nOnly a small number of indicators, such as the use of intrauterine devices and rate of C-section, increased during the pandemic. An increase in intrauterine device demand during the pandemic might be attributed to the likelihood of women seeking long-acting reversible contraceptives, which', 'changes of several reproductive and child health indicators assessed.']</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>According to the context, the following child health indicators improved despite the pandemic:
+1. **Pneumococcal conjugate vaccine** uptake, which increased by over 4 percentage points (Page 1).
+2. **Kangaroo mother care method** utilization, which increased from 8.6% to 10.4% (p &lt; 0.001) (Page 4).
+3. **Home visits/postnatal follow-up** during days 0–3, which increased from 36.8% to 40.0% (p &lt; 0.001) (Page 4).
+These indicators showed a statistically significant increase during the peri-COVID-19 pandemic period.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>Kangaroo mother care (8.6% to 10.4%) and home visits/postnatal follow-ups during days 0–3 (36.8% to 40.0%).</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>The child health indicators that improved despite the pandemic are:
-* Institutional live births beneficiaries of the kangaroo mother care method (increased from 8.6% to 10.4%, p &lt; 0.001)
-* Home visits/postnatal follow-up during days 0–3 (increased from 36.8% to 40.0%, p &lt; 0.001)
-* Pneumococcal conjugate vaccine (increased by over 4 percentage points)
-These indicators showed a statistically significant increase during the pandemic period, as stated in the text:
-* Page 4: "However, there were statistically significantly increases during the same period in the proportion of institutional live births beneficiaries of the kangaroo mother care method (from 8.6% to 10.4%, p &lt; 0.001) and home visits/postnatal follow-up during days 0–3 (from 36.8% to 40.0%, p &lt; 0.001)."
-* Page 1: "Likewise, the proportions of children who received ... pneumococcal conjugate vaccine increased by over 4 percentage points." 
-* Page 4: "in contrast, pneumococcal conjugate vaccine increased by over 4 percentage points."</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -693,30 +731,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>['partially account for the decline observed in RMNCAH services in Haiti.', 'Conclusions. The COVID-19 pandemic may have contributed to the decline observed in several RMNCAH indicators in Haiti. However, the role played by the sociopolitical crisis and control exercised by armed groups over the population in the last three years cannot be ruled out.\n\nKeywords\n\nChild health; family planning; maternal health; reproductive health; women’s health services; COVID-19; Haiti.', 'The COVID-19 pandemic came on top of a country already deeply affected by a sociopolitical and economic crisis, with a precarious healthcare system, and ravaged by corruption (20). , Haiti has been severely affected by political unrest, violent protests, national lockdowns, armed gang activities, and frequent kidnappings, all of which are frequently associ- ated with disruption in essential RMNCAH services.', 'in health services due to fear of contacting the virus and restrictions on movement, and closure of certain RMNCH services, among others (13, 14). Both of these are lower-middle-income coun- tries that might share similar obstacles in delivering sufficient services in times of crisis, comparable with Haiti. in contrast, Shikuku et al. (16), investigating the initial impact of COVID-19 pandemic on RMNCAH services in Kenya, found no significant change in the mean total hospital attendance. Nonetheless, the short period examined might be a possible explanation for the absence of significant impact of the COVID-19 pandemic on RMNCAH services in that study.', 'the SISNU–DHIS2 reporting sys- tem itself may have been negatively impacted by COVID-19, as well as the political turmoil and natural events that have affected Haiti.']</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Several external factors, besides COVID-19, may have influenced RMNCAH services in Haiti. These include:
+1. **Sociopolitical crisis**: The country has been experiencing a deep sociopolitical and economic crisis, which has led to a precarious healthcare system, corruption, and disruptions in essential RMNCAH services (Page 6).
+2. **Control exercised by armed groups**: Armed groups have been controlling parts of the population, which may have impacted the delivery of RMNCAH services (Page 1).
+3. **Political unrest and violent protests**: Frequent protests, national lockdowns, and violent unrest have been associated with disruptions in essential RMNCAH services (Page 6).
+4. **Armed gang activities and kidnappings**: These have contributed to the instability and disruptions in RMNCAH services (Page 6).
+5. **Natural events**: Haiti has been affected by natural events, which may have also impacted the SISNU–DHIS2 reporting system and RMNCAH services (Page 6).
+These factors may have partially accounted for the decline observed in RMNCAH services in Haiti, alongside the COVID-19 pandemic.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>The sociopolitical crisis and control of armed groups over populations, which disrupted healthcare access.</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>External factors, besides COVID-19, that may have influenced RMNCAH services in Haiti are:
-* Sociopolitical crisis
-* Control exercised by armed groups over the population
-* Economic crisis
-* Political unrest
-* Violent protests
-* National lockdowns
-* Armed gang activities
-* Frequent kidnappings
-* Corruption
-These factors are mentioned in the text as potentially contributing to the decline in RMNCAH services in Haiti, alongside the COVID-19 pandemic. (Page 1, 6) 
-The text explicitly states: "the role played by the sociopolitical crisis and control exercised by armed groups over the population in the last three years cannot be ruled out" (Page 1) and "Haiti has been severely affected by political unrest, violent protests, national lockdowns, armed gang activities, and frequent kidnappings, all of which are frequently associated with disruption in essential RMNCAH services." (Page 6)</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -726,24 +763,23 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>['The death of cardiac myocytes diminishes the heart’s pump function and is a major causes? of heart failure, one of the dominant causes? of death worldwide. Other than transplantation, there are no therapies that directly address the loss of cardiac myocytes, which explains the current excitement in cardiac regeneration. The ﬁeld is evolving in two important directions. First, although endogenous mammalian cardiac regeneration clearly seems to decline rapidly after birth, it may still persist in adulthood. The careful elucidation of the cellular and molecular mechanisms of endogenous heart regeneration may therefore provide an opportunity for develop- ing therapeutic interventions that amplify this process. Second, recent break- throughs have enabled reprogramming of cells that were apparently', 'There is reason for optimism for a regenerative medicine approach to heart failure, given the intense research efforts and the capacity of higher organisms, including the neonatal mouse, to regenerate myocardium. Perhaps the most important issue in this ﬁeld is identifying which ﬁndings are consistently supported by multiple experimental approaches. Ultimately, the ﬁndings that are easily repro- duced by most or all laboratories will most likely beneﬁt patients.\n\nThe authors declare that they have no conﬂict of interest.', 'Thus, there has been enormous interest in the prospect of cardiac regeneration rather than slowing the inexorable decline of heart function.\n\nUntil recently, the prospect of cardiac regeneration was largely a subject of science ﬁction. The longstanding paradigm held that the mammalian heart is a terminally differentiated organ, incapable of replenishing any myocyte attrition. During the past decade, however, studies revealed not only that mammalian cardiac myocytes retain some capacity for division (Beltrami et al, 2001), but also identiﬁed endogenous cardiac progenitor cells in the heart (Beltrami et al, 2003) or bone marrow (Orlic et al, 2001). These cells retain some potential for differentiation into the cellular components of the heart,', '|\n\nCardiovascular Diseases\n\nRegeneration of the heart\n\nMatthew L. Steinhauser1*, Richard T. Lee1,2**\n\nKeywords: cardiovascular disease; cardiac myocyte; heart failure; regeneration; stem cell\n\nDOI 10.1002/emmm.201100175\n\nReceived June 6, 2011 / Revised July 3, 2011 / Accepted August 1, 2011\n\nIntroduction', 'In light of mixed results from clinical trials, it is worth revisiting both the foundations of cardiac regeneration and highlight recent advances that may portend future directions in the ﬁeld. We will ﬁrst deﬁne the problem, that is elucidating the scope of endogenous mammalian regeneration and, by extension, the scale of the regenerative deﬁcit. We will then summarize current regenerative approaches, including both cell-based therapies and pharmacoregenerative strategies. in this context, we will summarize the many challenges that stand in the way of cardiac regeneration, both endogenous repair processes and exogenous regenerative therapies.']</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Heart regeneration is a major focus in medicine because the death of cardiac myocytes is a major cause of heart failure, which is one of the dominant causes of death worldwide. Currently, there are no therapies that directly address the loss of cardiac myocytes, except for transplantation. Therefore, researchers are excited about the potential of cardiac regeneration to provide new therapeutic interventions that can amplify the body's natural repair processes or replace damaged cells (Page 1, Document: regeneration).</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>Because loss of cardiac myocytes after events like myocardial infarction leads to heart failure, one of the top causes of death worldwide.</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Heart regeneration is a major focus in medicine because:
-* The death of cardiac myocytes (heart cells) leads to a decline in the heart's pump function, causing heart failure, which is a dominant cause of death worldwide.
-* Currently, there are no therapies that directly address the loss of cardiac myocytes, except for transplantation.
-* The potential for cardiac regeneration offers a new approach to treating heart failure, with research efforts focused on amplifying endogenous heart regeneration and developing therapeutic interventions.
-This is stated in the text: "The death of cardiac myocytes diminishes the heart’s pump function and is a major cause of heart failure, one of the dominant causes of death worldwide. Other than transplantation, there are no therapies that directly address the loss of cardiac myocytes, which explains the current excitement in cardiac regeneration." (Page 1) 
-Additionally, the text highlights the significance of cardiac regeneration as "there has been enormous interest in the prospect of cardiac regeneration rather than slowing the inexorable decline of heart function." (Page 1)</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -753,20 +789,23 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>['Evidence for heart regeneration in mammals', 'The regenerative deﬁcit of the mammalian heart is obvious when compared with organisms such as zebraﬁsh and newts, which demonstrate a remarkable survival capacity after removal of up to 20% of the heart by transection of the ventricular apex (Oberpriller &amp; Oberpriller, 1974; Poss et al, 2002). Pre-existing cardiac myocytes adjacent to the site appear to undergo a process of dedifferentiation, characterized by dissolution of sarcomeric structures. This is followed by incorporation of deoxyribonucleic acid (DNA) synthesis markers (e.g. nucleotide analogues) consistent with prolifera- tion (Jopling et al, 2010; Kikuchi et al, 2010; Laube et al, 2006). Ultimately, newly generated cardiac myocytes are functionally integrated with the preexisting myocardium. The heart is left with little', 'The data generated by these diverse methodologies support the notion that the mammalian heart has conserved some capacity for cardiac myocyte turnover though there is lingering con- troversy about the scope of the mammalian heart’s endogenous regenerativecapacity.Studiesrelyingontheidentiﬁcation mitotic cardiac myocytes (Kajstura et al, 1998), immuno-detection of cell cycle markers such as Ki67 (Beltrami et al, 2001) or of IdU incorporation into newly synthesized DNA(Kajstura et al, 2010b) suggest thatnearly 30% ofthe heart can bereplaced within 1 year during normal homeostasis, a rate that increases 50-fold after injury. These remarkably high rates imply that the entire heart is replaced approximately every 3 years during normal home-', 'The heart also presents a unique challenge compared to other organs owing to the propensity of cardiac myocytes to synthesize DNA during S-phase without completing either mitosis and/or cytokinesis (Fig 1). During early post-natal development, for example, the majority of rodent cardiac myocytes (Li et al, 1996) and an estimated 25–57% of human cardiac myocytes (Olivetti et al, 1996; Schmid &amp; Pﬁtzer, 1985) become binucleated. Byadulthood, most cardiacmyocyte nuclei have also become polyploid with at least one (4n: tetraploid) or two (8n: octoploid) additional rounds of chromosomal replication (Bergmann et al, 2010). Although some studies demonstratedthatthepolyploidyrateinthecardiacmyocytepool is not affected by ageing or injury (Olivetti et al, 1996), others suggested that the ploidy', 'Thus, there has been enormous interest in the prospect of cardiac regeneration rather than slowing the inexorable decline of heart function.\n\nUntil recently, the prospect of cardiac regeneration was largely a subject of science ﬁction. The longstanding paradigm held that the mammalian heart is a terminally differentiated organ, incapable of replenishing any myocyte attrition. During the past decade, however, studies revealed not only that mammalian cardiac myocytes retain some capacity for division (Beltrami et al, 2001), but also identiﬁed endogenous cardiac progenitor cells in the heart (Beltrami et al, 2003) or bone marrow (Orlic et al, 2001). These cells retain some potential for differentiation into the cellular components of the heart,']</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>The traditional belief about the mammalian heart was that it is a **terminally differentiated organ, incapable of replenishing any myocyte attrition** (Page 1). This longstanding paradigm held that the mammalian heart lacks the ability to regenerate or replace damaged cardiac myocytes.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
           <t>That it was a terminally differentiated organ incapable of regenerating lost myocytes.</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>The traditional belief about the mammalian heart was that it is a terminally differentiated organ, incapable of replenishing any myocyte attrition. 
-This is stated in the text: "Until recently, the prospect of cardiac regeneration was largely a subject of science ﬁction. The longstanding paradigm held that the mammalian heart is a terminally differentiated organ, incapable of replenishing any myocyte attrition." (Page 1)</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -776,27 +815,23 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>['www.embomolmed.org\n\nEMBO Mol Med 3, 701–712\n\nHeart regeneration in lower organisms', 'The regenerative deﬁcit of the mammalian heart is obvious when compared with organisms such as zebraﬁsh and newts, which demonstrate a remarkable survival capacity after removal of up to 20% of the heart by transection of the ventricular apex (Oberpriller &amp; Oberpriller, 1974; Poss et al, 2002). Pre-existing cardiac myocytes adjacent to the site appear to undergo a process of dedifferentiation, characterized by dissolution of sarcomeric structures. This is followed by incorporation of deoxyribonucleic acid (DNA) synthesis markers (e.g. nucleotide analogues) consistent with prolifera- tion (Jopling et al, 2010; Kikuchi et al, 2010; Laube et al, 2006). Ultimately, newly generated cardiac myocytes are functionally integrated with the preexisting myocardium. The heart is left with little', 'Evidence for heart regeneration in mammals', 'Orlic D, Kajstura J, Chimenti S, Jakoniuk I, Anderson SM, Li B, Pickel J, McKay R, Nadal-Ginard B, Bodine DM et al (2001) Bone marrow cells regenerate infarcted myocardium. Nature 410: 701-705\n\nPorrello ER, Mahmoud AI, Simpson E, Hill JA, Richardson JA, Olson EN, Sadek HA (2011) Transient regenerative potential of the neonatal mouse heart. Science 331: 1078-1080\n\nPoss KD, Wilson LG, Keating MT (2002) Heart regeneration in zebraﬁsh. Science 298: 2188-2190\n\nQuaini F, Urbanek K, Beltrami AP, Finato N, Beltrami CA, Nadal-Ginard B, Kajstura J, Leri A, Anversa P (2002) Chimerism of the transplanted heart. N Engl J Med 346: 5-15', 'Ieda M, Fu JD, Delgado-Olguin P, Vedantham V, Hayashi Y, Bruneau BG, Srivastava D (2010) Direct reprogramming of ﬁbroblasts into functional cardiomyocytes by deﬁned factors. Cell 142: 375-386\n\nJackson KA, Majka SM, Wang H, Pocius J, Hartley CJ, Majesky MW, Entman ML, Michael LH, Hirschi KK, Goodell MA (2001) Regeneration of ischemic cardiac muscle and vascular endothelium by adult stem cells. J Clin Invest 107: 1395-1402\n\nJopling C,Sleep E, Raya M, Marti M, Raya A, Belmonte JC(2010) Zebraﬁshheart regeneration occurs by cardiomyocyte dedifferentiation and proliferation. Nature 464: 606-609']</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Zebrafish and newts are lower organisms that show natural heart regeneration. They have been observed to have a remarkable survival capacity after removal of up to 20% of the heart, with pre-existing cardiac myocytes undergoing dedifferentiation, proliferation, and functional integration with the pre-existing myocardium (Oberpriller &amp; Oberpriller, 1974; Poss et al, 2002). Specifically, studies have shown that zebrafish can regenerate their heart through cardiomyocyte dedifferentiation and proliferation (Jopling et al, 2010; Poss et al, 2002).</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>Zebrafish and newts, which can regenerate up to 20% of their heart tissue after injury.</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Lower organisms that show natural heart regeneration include:
-* Zebrafish
-* Newts
-These organisms have been observed to have a remarkable survival capacity after removal of up to 20% of the heart, with pre-existing cardiac myocytes undergoing dedifferentiation, proliferation, and ultimately functional integration with the pre-existing myocardium (Oberpriller &amp; Oberpriller, 1974; Poss et al, 2002; Jopling et al, 2010). 
-References:
-- Oberpriller &amp; Oberpriller (1974)
-- Poss et al (2002)
-- Jopling et al (2010) 
-Page 2, 10.</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -806,28 +841,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>['The regenerative deﬁcit of the mammalian heart is obvious when compared with organisms such as zebraﬁsh and newts, which demonstrate a remarkable survival capacity after removal of up to 20% of the heart by transection of the ventricular apex (Oberpriller &amp; Oberpriller, 1974; Poss et al, 2002). Pre-existing cardiac myocytes adjacent to the site appear to undergo a process of dedifferentiation, characterized by dissolution of sarcomeric structures. This is followed by incorporation of deoxyribonucleic acid (DNA) synthesis markers (e.g. nucleotide analogues) consistent with prolifera- tion (Jopling et al, 2010; Kikuchi et al, 2010; Laube et al, 2006). Ultimately, newly generated cardiac myocytes are functionally integrated with the preexisting myocardium. The heart is left with little', 'Kikuchi K, Holdway JE, Werdich AA, Anderson RM, Fang Y, Egnaczyk GF, Evans T, Macrae CA, Stainier DY, Poss KD (2010) Primary contribution to zebraﬁsh heart regeneration by gata4(þ) cardiomyocytes. Nature 464: 601-605\n\nKolodziejczyk SM, Wang L, Balazsi K, DeRepentigny Y, Kothary R, Megeney LA (1999) MEF2 is upregulated during cardiac hypertrophy and is required for normal post-natal growth of the myocardium. Curr Biol 9: 1203-1206\n\n710', 'Ieda M, Fu JD, Delgado-Olguin P, Vedantham V, Hayashi Y, Bruneau BG, Srivastava D (2010) Direct reprogramming of ﬁbroblasts into functional cardiomyocytes by deﬁned factors. Cell 142: 375-386\n\nJackson KA, Majka SM, Wang H, Pocius J, Hartley CJ, Majesky MW, Entman ML, Michael LH, Hirschi KK, Goodell MA (2001) Regeneration of ischemic cardiac muscle and vascular endothelium by adult stem cells. J Clin Invest 107: 1395-1402\n\nJopling C,Sleep E, Raya M, Marti M, Raya A, Belmonte JC(2010) Zebraﬁshheart regeneration occurs by cardiomyocyte dedifferentiation and proliferation. Nature 464: 606-609', 'www.embomolmed.org\n\nEMBO Mol Med 3, 701–712\n\nHeart regeneration in lower organisms', 'the mitotic activity of mononucleated cardiac myocytes may provide an alternative approach to replenishing cardiac myocytes. A major concern with systemic growth factor therapy, however, is the potential for mitogenic effects that may impact other organs. Thus, the future of pharmacologic regeneration may lie in the local delivery of engineered proteins and small molecules that target speciﬁc survival, growth and differentiation pathways.\n\nPending issues\n\nDissect the mechanistic differences between adult mammals with limited regenerative capacity and organisms, such as neonatal mice, zebrafish and newts, that demonstrate unambiguous cardiac myocyte regeneration. Understanding these differences may reveal new pathways that can be therapeutically targeted to achieve more robust regeneration.']</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Zebrafish heart regeneration occurs through the following mechanisms:
+1. **Dedifferentiation**: Pre-existing cardiac myocytes adjacent to the injury site undergo dedifferentiation, characterized by the dissolution of sarcomeric structures.
+2. **Proliferation**: Dedifferentiated cardiac myocytes then undergo DNA synthesis and proliferation, as evidenced by the incorporation of DNA synthesis markers.
+3. **Functional integration**: Newly generated cardiac myocytes are functionally integrated with the pre-existing myocardium.
+According to studies, gata4(+) cardiomyocytes are the primary contributors to zebrafish heart regeneration (Kikuchi et al, 2010). Additionally, research has shown that zebrafish heart regeneration occurs through cardiomyocyte dedifferentiation and proliferation (Jopling et al, 2010).</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>Dedifferentiation of pre-existing cardiomyocytes followed by proliferation and reintegration into the myocardium.</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>The mechanisms underlying zebrafish heart regeneration involve:
-1. Dedifferentiation of pre-existing cardiac myocytes adjacent to the injury site, characterized by dissolution of sarcomeric structures.
-2. Proliferation of these dedifferentiated cardiac myocytes, as evidenced by incorporation of DNA synthesis markers.
-3. Functional integration of newly generated cardiac myocytes with the pre-existing myocardium.
-Studies have shown that gata4(+) cardiomyocytes make a primary contribution to zebrafish heart regeneration (Kikuchi et al, 2010). Additionally, research has demonstrated that zebrafish heart regeneration occurs through cardiomyocyte dedifferentiation and proliferation (Jopling et al, 2010).
-References:
-- Jopling et al (2010)
-- Kikuchi et al (2010) 
-- Oberpriller &amp; Oberpriller (1974)
-- Poss et al (2002)</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -837,32 +871,35 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>['Evidence for heart regeneration in mammals', 'The regenerative deﬁcit of the mammalian heart is obvious when compared with organisms such as zebraﬁsh and newts, which demonstrate a remarkable survival capacity after removal of up to 20% of the heart by transection of the ventricular apex (Oberpriller &amp; Oberpriller, 1974; Poss et al, 2002). Pre-existing cardiac myocytes adjacent to the site appear to undergo a process of dedifferentiation, characterized by dissolution of sarcomeric structures. This is followed by incorporation of deoxyribonucleic acid (DNA) synthesis markers (e.g. nucleotide analogues) consistent with prolifera- tion (Jopling et al, 2010; Kikuchi et al, 2010; Laube et al, 2006). Ultimately, newly generated cardiac myocytes are functionally integrated with the preexisting myocardium. The heart is left with little', 'Orlic D, Kajstura J, Chimenti S, Jakoniuk I, Anderson SM, Li B, Pickel J, McKay R, Nadal-Ginard B, Bodine DM et al (2001) Bone marrow cells regenerate infarcted myocardium. Nature 410: 701-705\n\nPorrello ER, Mahmoud AI, Simpson E, Hill JA, Richardson JA, Olson EN, Sadek HA (2011) Transient regenerative potential of the neonatal mouse heart. Science 331: 1078-1080\n\nPoss KD, Wilson LG, Keating MT (2002) Heart regeneration in zebraﬁsh. Science 298: 2188-2190\n\nQuaini F, Urbanek K, Beltrami AP, Finato N, Beltrami CA, Nadal-Ginard B, Kajstura J, Leri A, Anversa P (2002) Chimerism of the transplanted heart. N Engl J Med 346: 5-15', 'www.embomolmed.org\n\nEMBO Mol Med 3, 701–712\n\nHeart regeneration in lower organisms', 'The data generated by these diverse methodologies support the notion that the mammalian heart has conserved some capacity for cardiac myocyte turnover though there is lingering con- troversy about the scope of the mammalian heart’s endogenous regenerativecapacity.Studiesrelyingontheidentiﬁcation mitotic cardiac myocytes (Kajstura et al, 1998), immuno-detection of cell cycle markers such as Ki67 (Beltrami et al, 2001) or of IdU incorporation into newly synthesized DNA(Kajstura et al, 2010b) suggest thatnearly 30% ofthe heart can bereplaced within 1 year during normal homeostasis, a rate that increases 50-fold after injury. These remarkably high rates imply that the entire heart is replaced approximately every 3 years during normal home-']</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>There is limited evidence suggesting that the mammalian heart has some capacity for cardiac myocyte turnover. Studies have reported:
+1. Presence of mitotic cardiac myocytes (Kajstura et al, 1998)
+2. Immuno-detection of cell cycle markers such as Ki67 (Beltrami et al, 2001)
+3. IdU incorporation into newly synthesized DNA (Kajstura et al, 2010b)
+These findings imply that nearly 30% of the heart can be replaced within 1 year during normal homeostasis, with a 50-fold increase after injury. However, there is still controversy about the scope of the mammalian heart's endogenous regenerative capacity.
+Notably, research in neonatal mice has shown a transient regenerative potential (Porrello et al, 2011). Additionally, some studies have suggested that bone marrow cells can contribute to myocardial regeneration (Orlic et al, 2001).
+However, it is essential to note that the regenerative capacity of the mammalian heart is still not well understood and appears to be much lower compared to lower organisms like zebrafish and newts. 
+References:
+- Kajstura et al, 1998
+- Beltrami et al, 2001
+- Kajstura et al, 2010b
+- Porrello et al, 2011
+- Orlic et al, 2001</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>Yes, neonatal mice can regenerate myocardium within the first week of life, but this capacity diminishes in adulthood.</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>There is limited evidence suggesting that the mammalian heart has some capacity for cardiac myocyte turnover and regeneration, but the scope of this capacity is still a topic of controversy.
- Studies have reported:
-* The presence of mitotic cardiac myocytes (Kajstura et al, 1998)
-* Immuno-detection of cell cycle markers such as Ki67 (Beltrami et al, 2001)
-* IdU incorporation into newly synthesized DNA (Kajstura et al, 2010b)
-These findings imply that nearly 30% of the heart can be replaced within 1 year during normal homeostasis, a rate that increases 50-fold after injury. However, it is unclear if this regenerative capacity is sufficient for complete heart regeneration.
-Additionally, some studies have shown that neonatal mouse hearts have a transient regenerative potential (Porrello et al, 2011). There is also evidence that bone marrow cells can contribute to myocardial regeneration (Orlic et al, 2001).
-However, more research is needed to fully understand the extent of heart regeneration in mammals.
-References:
-- Kajstura et al (1998)
-- Beltrami et al (2001)
-- Kajstura et al (2010b)
-- Porrello et al (2011)
-- Orlic et al (2001)</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -872,28 +909,31 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>['progenitors was rapidly translated into the clinic to treat human ischemic heart disease. A number of randomized trials, using bone marrow mononuclear cells have been performed and most studies demonstrated modest cell therapy-mediated improve- ments in ventricular function. in the largest study to date, the reinfusion of enriched progenitor cells and infarct remodeling in AMI (REPAIR-AMI) study (Schachinger et al, 2006), 204 randomized patients with acute myocardial infarctions received intracoronary delivery of bone marrow cells or vehicle control. Follow-up after 1 year demonstrated signiﬁcant improvements in both cardiac function and in a combined clinical endpoint consisting of death, recurrent myocardial infarct or any revascularization procedure. in contrast, analysis of 18-month', 'If progenitor cells residing in the adult are capable of producing new heart cells, the therapeutic delivery of such progenitors might facilitate the generation of de novo functional myocardium. in this context, cell-based therapies for the heart have been rapidly translated into the clinic to treat heart disease, but randomized clinical trials with bone marrow progenitors have shown at best modest improvements in ventricular function (Martin-Rendon et al, 2008). in short, the promise of complete cardiac regeneration has not yet been realized.', 'Nonetheless, some therapeutic effect was observed even in studies with no detectable transdifferentiation (Balsam et al, 2004). Cell-based therapy using autologous bone marrow\n\nExogenous cell-based therapy O = OO = O O = O O=O O=O Ischemia Endogenous stem cell niche Homing Proliferation Differentiation Inflammation Myocyte deficit ~ 1 billion cells Paracrine factors D i visio n Fibrosis', 'bone marrow mononuclear cells: patients experience modest improvements in ventricular function with subtle improvements in heart failure symptoms. Overall, the experi- ence with cell-basedtherapies inhumans does notsupport wide- spread adoption at this time given their modest beneﬁts, insufﬁcient safety data and the anticipated quality control costs of bringing these therapies to the bedside.', 'other contemporaneous studies suggested that the source of circulating progenitors could be the bone marrow. in both cases, a bone marrow cell population with a higher density of the cell surface receptor c-kit, showed repopulation of murine cardiac myocytes after experimental myocardial infarction (Jackson et al, 2001; Orlic et al, 2001). Since these initial reports, a number of studies failed to demonstrate similar rates of chimerism in transplanted hearts (Deb et al, 2003; Hocht-Zeisberg et al, 2004; Laﬂamme et al, 2002; Muller et al, 2002) or potency of bone marrow stem cells (Balsam et al, 2004; Murry et al, 2004) leading some to postulate that cardiac myocyte transdifferentiation was overestimated owing to an artefact (Laﬂamme &amp; Murry, 2005).']</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>The outcome of cell-based therapies with bone marrow progenitors has shown modest improvements in ventricular function and subtle improvements in heart failure symptoms. 
+Key findings:
+- Randomized trials using bone marrow mononuclear cells have demonstrated modest cell therapy-mediated improvements in ventricular function (Martin-Rendon et al, 2008; Schachinger et al, 2006).
+- The REPAIR-AMI study (Schachinger et al, 2006) showed significant improvements in cardiac function and a combined clinical endpoint.
+- However, the benefits are limited, and there is insufficient safety data to support widespread adoption (Balsam et al, 2004; Martin-Rendon et al, 2008).
+References:
+- Schachinger et al, 2006
+- Martin-Rendon et al, 2008
+- Balsam et al, 2004</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>They showed only modest improvements in ventricular function, falling short of complete regeneration.</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>The outcome of cell-based therapies with bone marrow progenitors has shown modest improvements in ventricular function and heart failure symptoms. 
-Studies have reported:
-* Modest cell therapy-mediated improvements in ventricular function (Martin-Rendon et al, 2008)
-* Significant improvements in cardiac function and a combined clinical endpoint in the REPAIR-AMI study (Schachinger et al, 2006)
-* Some therapeutic effect observed even in studies with no detectable transdifferentiation (Balsam et al, 2004)
-However, the benefits are limited, and there are concerns regarding safety, quality control, and cost. As a result, widespread adoption of these therapies is not currently supported.
-References:
-- Martin-Rendon et al (2008)
-- Schachinger et al (2006)
-- Balsam et al (2004)</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -903,25 +943,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>['Ieda M, Fu JD, Delgado-Olguin P, Vedantham V, Hayashi Y, Bruneau BG, Srivastava D (2010) Direct reprogramming of ﬁbroblasts into functional cardiomyocytes by deﬁned factors. Cell 142: 375-386\n\nJackson KA, Majka SM, Wang H, Pocius J, Hartley CJ, Majesky MW, Entman ML, Michael LH, Hirschi KK, Goodell MA (2001) Regeneration of ischemic cardiac muscle and vascular endothelium by adult stem cells. J Clin Invest 107: 1395-1402\n\nJopling C,Sleep E, Raya M, Marti M, Raya A, Belmonte JC(2010) Zebraﬁshheart regeneration occurs by cardiomyocyte dedifferentiation and proliferation. Nature 464: 606-609', 'also expressed by non-cardiovascular cells/progenitors or because they may be part of the stress-induced reactivation of ‘foetal gene programmes’, a phenomenon that is well documented in adult cardiac myocytes (Bisping et al, 2006; Kolodziejczyk et al, 1999; Saadane et al, 1999).\n\nMoving towards a regenerative therapy', 'In this review, we have described the current status of research on cardiac regeneration, highlighting important recent discoveries and ongoing controversies. The initial hope that a cell progenitor would emerge with the capacity to regenerate the injured mammalian heart in the same manner that bone marrow may be reconstituted has not been realized in animal studies or randomized clinical studies. Even if some studies have questioned the regenerative potency of various endogenous progenitor populations, it is clearly feasible to reprogramme many cell types to differentiate into cardiomyocytes. Interestingly, evolving notions of cellular plasticity may ultimately help to explain the frustration that many in the ﬁeld have experienced when attempting to replicate the ﬁndings of landmark', 'A more realistic short-term goal may be to exploit paracrine signalling to amplify the existent endogenous regenerative response. Recent cell transplantation experiments conducted in our laboratory, using an inducible cre-based genetic lineage mapping approach, tested the hypothesis that cell-based therapies might exert proregenerative effects via a paracrine mechanism (Loffredo et al, 2011) (Fig 5). Consistent with some prior studies (Balsam et al, 2004; Murry et al, 2004), we found no evidence for transdifferentiation of exogenously delivered bone marrow cells into cardiac myocytes. However, we did ﬁnd increased generation of cardiac myocytes from endogenous progenitors in mice, which were administered c-kitþ bone marrow cells but not mesenchymal stem cells. This ﬁnding suggests', 'Complete molecular and functional characterization of endogenous cardiac myocyte progenitors. Multiple laboratories have isolated progenitors from the heart with different molecular characteristics. What are the in vivo functional roles of these progenitors? Do the observed molecular differences between these isolated cells represent functionally distinct cell types?\n\nIdentify paracrine signalling pathways responsible for activation and recruitment of endogenous cardiac myocyte progenitors. This may facilitate a pharmacoregenerative therapy, in which treatment with a protein or small molecule would hold the promise of amplifying endogenous regeneration.']</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Cellular reprogramming plays a significant role in regeneration, particularly in cardiac regeneration. Research has shown that it is feasible to reprogram many cell types to differentiate into cardiomyocytes (Ieda et al, 2010). 
+Key findings:
+- Direct reprogramming of fibroblasts into functional cardiomyocytes by defined factors has been achieved (Ieda et al, 2010).
+- Cellular reprogramming offers a promising approach to amplify endogenous regeneration, potentially through paracrine signalling pathways (Loffredo et al, 2011).
+However, further research is needed to fully understand the role of cellular reprogramming in regeneration and to explore its therapeutic potential. 
+References:
+- Ieda et al, 2010
+- Loffredo et al, 2011</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>Cells like fibroblasts can be reprogrammed into cardiomyocytes, showing potential for regenerative therapy.</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Cellular reprogramming plays a significant role in regeneration, particularly in the context of cardiac regeneration. 
-Studies have shown that cellular reprogramming can be used to directly convert non-cardiac cells into functional cardiomyocytes. For example, Ieda et al (2010) demonstrated that fibroblasts can be reprogrammed into functional cardiomyocytes by defined factors. 
-This approach holds promise for regenerative therapies, as it may be possible to reprogram non-cardiac cells to replace damaged or lost cardiac tissue. Additionally, cellular reprogramming may also be used to activate endogenous cardiac progenitor cells, which can then contribute to the regeneration of cardiac tissue.
-However, further research is needed to fully understand the role of cellular reprogramming in regeneration and to translate these findings into clinical therapies.
-References:
-- Ieda M, Fu JD, Delgado-Olguin P, Vedantham V, Hayashi Y, Bruneau BG, Srivastava D (2010) 
-- Jopling C, Sleep E, Raya M, Marti M, Raya A, Belmonte JC (2010)</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -931,25 +976,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>['In light of mixed results from clinical trials, it is worth revisiting both the foundations of cardiac regeneration and highlight recent advances that may portend future directions in the ﬁeld. We will ﬁrst deﬁne the problem, that is elucidating the scope of endogenous mammalian regeneration and, by extension, the scale of the regenerative deﬁcit. We will then summarize current regenerative approaches, including both cell-based therapies and pharmacoregenerative strategies. in this context, we will summarize the many challenges that stand in the way of cardiac regeneration, both endogenous repair processes and exogenous regenerative therapies.', 'the mitotic activity of mononucleated cardiac myocytes may provide an alternative approach to replenishing cardiac myocytes. A major concern with systemic growth factor therapy, however, is the potential for mitogenic effects that may impact other organs. Thus, the future of pharmacologic regeneration may lie in the local delivery of engineered proteins and small molecules that target speciﬁc survival, growth and differentiation pathways.\n\nPending issues\n\nDissect the mechanistic differences between adult mammals with limited regenerative capacity and organisms, such as neonatal mice, zebrafish and newts, that demonstrate unambiguous cardiac myocyte regeneration. Understanding these differences may reveal new pathways that can be therapeutically targeted to achieve more robust regeneration.', 'The death of cardiac myocytes diminishes the heart’s pump function and is a major causes? of heart failure, one of the dominant causes? of death worldwide. Other than transplantation, there are no therapies that directly address the loss of cardiac myocytes, which explains the current excitement in cardiac regeneration. The ﬁeld is evolving in two important directions. First, although endogenous mammalian cardiac regeneration clearly seems to decline rapidly after birth, it may still persist in adulthood. The careful elucidation of the cellular and molecular mechanisms of endogenous heart regeneration may therefore provide an opportunity for develop- ing therapeutic interventions that amplify this process. Second, recent break- throughs have enabled reprogramming of cells that were apparently', 'Thus, there has been enormous interest in the prospect of cardiac regeneration rather than slowing the inexorable decline of heart function.\n\nUntil recently, the prospect of cardiac regeneration was largely a subject of science ﬁction. The longstanding paradigm held that the mammalian heart is a terminally differentiated organ, incapable of replenishing any myocyte attrition. During the past decade, however, studies revealed not only that mammalian cardiac myocytes retain some capacity for division (Beltrami et al, 2001), but also identiﬁed endogenous cardiac progenitor cells in the heart (Beltrami et al, 2003) or bone marrow (Orlic et al, 2001). These cells retain some potential for differentiation into the cellular components of the heart,', 'In this review, we have described the current status of research on cardiac regeneration, highlighting important recent discoveries and ongoing controversies. The initial hope that a cell progenitor would emerge with the capacity to regenerate the injured mammalian heart in the same manner that bone marrow may be reconstituted has not been realized in animal studies or randomized clinical studies. Even if some studies have questioned the regenerative potency of various endogenous progenitor populations, it is clearly feasible to reprogramme many cell types to differentiate into cardiomyocytes. Interestingly, evolving notions of cellular plasticity may ultimately help to explain the frustration that many in the ﬁeld have experienced when attempting to replicate the ﬁndings of landmark']</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>The major barriers to successful cardiac regeneration in humans include:
+1. **Limited understanding of endogenous mammalian regeneration**: The scope of endogenous mammalian regeneration and the scale of the regenerative deficit are not well understood.
+2. **Mechanistic differences between adult mammals and organisms with high regenerative capacity**: The differences between adult mammals with limited regenerative capacity and organisms like neonatal mice, zebrafish, and newts that demonstrate unambiguous cardiac myocyte regeneration are not well understood.
+3. **Challenges in cell-based therapies**: Cell-based therapies have shown modest improvements in ventricular function and heart failure symptoms, but the benefits are limited, and there is insufficient safety data to support widespread adoption.
+4. **Limited cardiac myocyte regeneration capacity**: The mammalian heart has a limited capacity for cardiac myocyte turnover, and this capacity declines rapidly after birth.
+Further research is needed to overcome these barriers and to develop effective therapeutic interventions for cardiac regeneration. 
+References: 
+- Multiple documents in the context ( scores: 0.8397080302238464,  0.8344274163246155,  0.8341291546821594,  0.8323609828948975,  0.8236168622970581)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>Limited regenerative capacity in adult mammals, poor reproducibility of some studies, and challenges in functional integration of new cells.</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>The major barriers to successful cardiac regeneration in humans include:
-1. **Limited understanding of endogenous mammalian regeneration**: Dissecting the mechanistic differences between adult mammals with limited regenerative capacity and organisms with robust cardiac regeneration (e.g., neonatal mice, zebrafish, and newts) is crucial.
-2. **Decline of endogenous cardiac regeneration after birth**: Endogenous mammalian cardiac regeneration seems to decline rapidly after birth, making it challenging to amplify this process therapeutically.
-3. **Limited potency of endogenous progenitor populations**: The regenerative potency of various endogenous progenitor populations has been questioned, and their ability to regenerate the injured mammalian heart has not been realized in animal studies or clinical trials.
-4. **Safety concerns and limited efficacy of cell-based therapies**: Cell-based therapies have shown modest improvements in ventricular function and heart failure symptoms, but their benefits are limited, and there are concerns regarding safety, quality control, and cost.
-5. **Need for targeted and efficient therapeutic interventions**: The development of therapeutic interventions that can specifically target survival, growth, and differentiation pathways to achieve more robust regeneration is necessary.
-These challenges highlight the complexity of cardiac regeneration and the need for further research to overcome these barriers and develop effective therapeutic strategies.</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -959,28 +1009,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>['In light of mixed results from clinical trials, it is worth revisiting both the foundations of cardiac regeneration and highlight recent advances that may portend future directions in the ﬁeld. We will ﬁrst deﬁne the problem, that is elucidating the scope of endogenous mammalian regeneration and, by extension, the scale of the regenerative deﬁcit. We will then summarize current regenerative approaches, including both cell-based therapies and pharmacoregenerative strategies. in this context, we will summarize the many challenges that stand in the way of cardiac regeneration, both endogenous repair processes and exogenous regenerative therapies.', 'A more realistic short-term goal may be to exploit paracrine signalling to amplify the existent endogenous regenerative response. Recent cell transplantation experiments conducted in our laboratory, using an inducible cre-based genetic lineage mapping approach, tested the hypothesis that cell-based therapies might exert proregenerative effects via a paracrine mechanism (Loffredo et al, 2011) (Fig 5). Consistent with some prior studies (Balsam et al, 2004; Murry et al, 2004), we found no evidence for transdifferentiation of exogenously delivered bone marrow cells into cardiac myocytes. However, we did ﬁnd increased generation of cardiac myocytes from endogenous progenitors in mice, which were administered c-kitþ bone marrow cells but not mesenchymal stem cells. This ﬁnding suggests', 'If progenitor cells residing in the adult are capable of producing new heart cells, the therapeutic delivery of such progenitors might facilitate the generation of de novo functional myocardium. in this context, cell-based therapies for the heart have been rapidly translated into the clinic to treat heart disease, but randomized clinical trials with bone marrow progenitors have shown at best modest improvements in ventricular function (Martin-Rendon et al, 2008). in short, the promise of complete cardiac regeneration has not yet been realized.', 'the mitotic activity of mononucleated cardiac myocytes may provide an alternative approach to replenishing cardiac myocytes. A major concern with systemic growth factor therapy, however, is the potential for mitogenic effects that may impact other organs. Thus, the future of pharmacologic regeneration may lie in the local delivery of engineered proteins and small molecules that target speciﬁc survival, growth and differentiation pathways.\n\nPending issues\n\nDissect the mechanistic differences between adult mammals with limited regenerative capacity and organisms, such as neonatal mice, zebrafish and newts, that demonstrate unambiguous cardiac myocyte regeneration. Understanding these differences may reveal new pathways that can be therapeutically targeted to achieve more robust regeneration.', 'Circumventing cell-based therapy with pharmacoregeneration?\n\nIt is hard to imagine that a single pharmacologic intervention could leads? to complete cardiac repair, but a number of recent discoveries lend credence to the underlying concept that paracrine signals may activate repair mechanisms in the heart. in general, the development of small molecule or protein-based therapies raises relatively modest problems with quality control compared to cell-based therapies. Therefore, pharmacoregen- erative approaches may be a more practical near-term approach to promote cardiac repair.']</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Promising directions for regenerative therapy include:
+1. **Exploiting paracrine signalling**: Amplifying the existent endogenous regenerative response through paracrine signalling pathways (Loffredo et al, 2011).
+2. **Pharmacoregenerative strategies**: Developing small molecule or protein-based therapies that target specific survival, growth, and differentiation pathways, potentially through local delivery of engineered proteins and small molecules (Document: regeneration, Score: 0.790810763835907).
+3. **Cell-based therapies with improved understanding**: Continuing to investigate cell-based therapies, understanding their limitations, and exploring ways to improve their efficacy, such as identifying the optimal cell type and delivery method.
+These directions aim to overcome the challenges in cardiac regeneration and provide new avenues for therapeutic interventions. 
+References:
+- Loffredo et al, 2011
+- Document: regeneration ( Scores: 0.8117988109588623,  0.8098053932189941,  0.7943543195724487,  0.7932941317558289,  0.790810763835907)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>Pharmacoregenerative strategies, local delivery of engineered proteins, small molecules targeting growth pathways, and refined reprogramming methods.</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Promising directions for regenerative therapy include:
-1. **Exploiting paracrine signalling**: Amplifying the existent endogenous regenerative response through paracrine signalling, which may activate repair mechanisms in the heart (Loffredo et al, 2011).
-2. **Pharmacoregenerative strategies**: Developing small molecule or protein-based therapies that target specific survival, growth, and differentiation pathways to achieve more robust regeneration (Martin-Rendon et al, 2008).
-3. **Local delivery of engineered proteins and small molecules**: Targeting specific pathways to promote cardiac repair while minimizing systemic side effects.
-4. **Understanding mechanistic differences between regenerative and non-regenerative organisms**: Dissecting the differences between adult mammals with limited regenerative capacity and organisms with robust cardiac regeneration to reveal new therapeutic targets.
-These approaches may offer more practical and efficient solutions for cardiac regeneration, addressing the limitations and challenges associated with cell-based therapies. 
-References:
-- Loffredo et al (2011)
-- Martin-Rendon et al (2008) 
-- Balsam et al (2004)</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -990,21 +1042,27 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>['In light of mixed results from clinical trials, it is worth revisiting both the foundations of cardiac regeneration and highlight recent advances that may portend future directions in the ﬁeld. We will ﬁrst deﬁne the problem, that is elucidating the scope of endogenous mammalian regeneration and, by extension, the scale of the regenerative deﬁcit. We will then summarize current regenerative approaches, including both cell-based therapies and pharmacoregenerative strategies. in this context, we will summarize the many challenges that stand in the way of cardiac regeneration, both endogenous repair processes and exogenous regenerative therapies.', 'There is reason for optimism for a regenerative medicine approach to heart failure, given the intense research efforts and the capacity of higher organisms, including the neonatal mouse, to regenerate myocardium. Perhaps the most important issue in this ﬁeld is identifying which ﬁndings are consistently supported by multiple experimental approaches. Ultimately, the ﬁndings that are easily repro- duced by most or all laboratories will most likely beneﬁt patients.\n\nThe authors declare that they have no conﬂict of interest.', 'the mitotic activity of mononucleated cardiac myocytes may provide an alternative approach to replenishing cardiac myocytes. A major concern with systemic growth factor therapy, however, is the potential for mitogenic effects that may impact other organs. Thus, the future of pharmacologic regeneration may lie in the local delivery of engineered proteins and small molecules that target speciﬁc survival, growth and differentiation pathways.\n\nPending issues\n\nDissect the mechanistic differences between adult mammals with limited regenerative capacity and organisms, such as neonatal mice, zebrafish and newts, that demonstrate unambiguous cardiac myocyte regeneration. Understanding these differences may reveal new pathways that can be therapeutically targeted to achieve more robust regeneration.', 'Thus, there has been enormous interest in the prospect of cardiac regeneration rather than slowing the inexorable decline of heart function.\n\nUntil recently, the prospect of cardiac regeneration was largely a subject of science ﬁction. The longstanding paradigm held that the mammalian heart is a terminally differentiated organ, incapable of replenishing any myocyte attrition. During the past decade, however, studies revealed not only that mammalian cardiac myocytes retain some capacity for division (Beltrami et al, 2001), but also identiﬁed endogenous cardiac progenitor cells in the heart (Beltrami et al, 2003) or bone marrow (Orlic et al, 2001). These cells retain some potential for differentiation into the cellular components of the heart,', 'The death of cardiac myocytes diminishes the heart’s pump function and is a major causes? of heart failure, one of the dominant causes? of death worldwide. Other than transplantation, there are no therapies that directly address the loss of cardiac myocytes, which explains the current excitement in cardiac regeneration. The ﬁeld is evolving in two important directions. First, although endogenous mammalian cardiac regeneration clearly seems to decline rapidly after birth, it may still persist in adulthood. The careful elucidation of the cellular and molecular mechanisms of endogenous heart regeneration may therefore provide an opportunity for develop- ing therapeutic interventions that amplify this process. Second, recent break- throughs have enabled reprogramming of cells that were apparently']</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>The most pressing issue for advancing cardiac regeneration research is **identifying which findings are consistently supported by multiple experimental approaches** (Score: 0.8298471570014954). This is crucial to ensure that the results are reliable and can be translated into therapeutic interventions that benefit patients.
+Additionally, understanding the **mechanistic differences between adult mammals with limited regenerative capacity and organisms with high regenerative capacity** (Score: 0.8267030715942383) is also a significant issue that needs to be addressed to reveal new pathways that can be therapeutically targeted to achieve more robust regeneration.
+Furthermore, **elucidating the scope of endogenous mammalian regeneration and the scale of the regenerative deficit** (Score: 0.8378692865371704) is also a pressing issue, as it is essential to understand the problem before developing effective therapeutic interventions. 
+References:
+- Document: regeneration (Scores: 0.8298471570014954, 0.8378692865371704, 0.8267030715942383)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
           <t>Identifying findings that are reproducible across laboratories, ensuring consistency and reliability before clinical translation.</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>The most pressing issue for advancing cardiac regeneration research is **identifying consistently supported findings across multiple experimental approaches**. This is crucial to ensure that research findings are reproducible and can be translated into therapeutic interventions that benefit patients.
-According to the context, "Perhaps the most important issue in this field is identifying which findings are consistently supported by multiple experimental approaches. Ultimately, the findings that are easily reproduced by most or all laboratories will most likely benefit patients." (Score: 0.8298471570014954)
-Additionally, understanding the mechanistic differences between adult mammals with limited regenerative capacity and organisms with robust cardiac regeneration is also a significant challenge that needs to be addressed (Score: 0.8267030715942383).</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>